<commit_message>
Q425 Earnings Season pt.1
</commit_message>
<xml_diff>
--- a/Financial Analysis/ADUI.xlsx
+++ b/Financial Analysis/ADUI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antos\Documents\GitHub\FinanceModels\Financial Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A9F70E-C822-4E0A-A6FC-0ADFE0821F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F4A49FE-37F9-4199-A4D2-31C14F312849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{4D8E8F3E-1FCF-429E-A59B-D9E70D9369D6}"/>
   </bookViews>
@@ -129,7 +129,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="[$$-409]#,##0.00"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -215,7 +215,7 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="4" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -628,7 +628,7 @@
       </c>
       <c r="F3" s="4">
         <f ca="1">TODAY()</f>
-        <v>45955</v>
+        <v>45983</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
@@ -1516,47 +1516,47 @@
         <v>2</v>
       </c>
       <c r="E12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" ref="E12:O12" si="7">420+(650-420)</f>
         <v>650</v>
       </c>
       <c r="F12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="G12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="H12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="I12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="J12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="K12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="L12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="M12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="N12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
       <c r="O12" s="5">
-        <f>420+(650-420)</f>
+        <f t="shared" si="7"/>
         <v>650</v>
       </c>
     </row>
@@ -1569,43 +1569,43 @@
         <v>0.15</v>
       </c>
       <c r="F13" s="7">
-        <f t="shared" ref="F13:O13" si="7">F11/F12</f>
+        <f t="shared" ref="F13:O13" si="8">F11/F12</f>
         <v>0.23423076923076927</v>
       </c>
       <c r="G13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.35134615384615386</v>
       </c>
       <c r="H13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.50593846153846156</v>
       </c>
       <c r="I13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.69882750000000016</v>
       </c>
       <c r="J13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>0.96191550000000003</v>
       </c>
       <c r="K13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.319961825</v>
       </c>
       <c r="L13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.7159503725000003</v>
       </c>
       <c r="M13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>2.2307354842500002</v>
       </c>
       <c r="N13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>2.8999561295250005</v>
       </c>
       <c r="O13" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>3.7699429683825003</v>
       </c>
     </row>
@@ -1622,43 +1622,43 @@
         <v>0.5</v>
       </c>
       <c r="F15" s="9">
-        <f t="shared" ref="F15:O15" si="8">F5/E5-1</f>
+        <f t="shared" ref="F15:O15" si="9">F5/E5-1</f>
         <v>0.44999999999999996</v>
       </c>
       <c r="G15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.39999999999999991</v>
       </c>
       <c r="H15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.35000000000000009</v>
       </c>
       <c r="I15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="J15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="K15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="L15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="M15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
       <c r="N15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.29999999999999982</v>
       </c>
       <c r="O15" s="9">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>0.30000000000000004</v>
       </c>
     </row>
@@ -1671,43 +1671,43 @@
         <v>0.42499999999999999</v>
       </c>
       <c r="F16" s="9">
-        <f t="shared" ref="F16:O16" si="9">F7/F5</f>
+        <f t="shared" ref="F16:O16" si="10">F7/F5</f>
         <v>0.43</v>
       </c>
       <c r="G16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.435</v>
       </c>
       <c r="H16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.44</v>
       </c>
       <c r="I16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.44500000000000006</v>
       </c>
       <c r="J16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.45</v>
       </c>
       <c r="K16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.45</v>
       </c>
       <c r="L16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.45</v>
       </c>
       <c r="M16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.45</v>
       </c>
       <c r="N16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.45</v>
       </c>
       <c r="O16" s="9">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>0.45</v>
       </c>
       <c r="Q16" s="1" t="s">
@@ -1726,43 +1726,43 @@
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="F17" s="9">
-        <f t="shared" ref="F17:O17" si="10">F9/F5</f>
+        <f t="shared" ref="F17:O17" si="11">F9/F5</f>
         <v>0.09</v>
       </c>
       <c r="G17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.1</v>
       </c>
       <c r="H17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.11</v>
       </c>
       <c r="I17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.12</v>
       </c>
       <c r="J17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.125</v>
       </c>
       <c r="K17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.125</v>
       </c>
       <c r="L17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.125</v>
       </c>
       <c r="M17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.125</v>
       </c>
       <c r="N17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.125</v>
       </c>
       <c r="O17" s="9">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>0.125</v>
       </c>
       <c r="Q17" s="1" t="s">
@@ -1781,43 +1781,43 @@
         <v>6.5000000000000002E-2</v>
       </c>
       <c r="F18" s="9">
-        <f t="shared" ref="F18:O18" si="11">F11/F5</f>
+        <f t="shared" ref="F18:O18" si="12">F11/F5</f>
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="G18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>7.4999999999999997E-2</v>
       </c>
       <c r="H18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.08</v>
       </c>
       <c r="I18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>8.5000000000000006E-2</v>
       </c>
       <c r="J18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>0.09</v>
       </c>
       <c r="K18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="L18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="M18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="N18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="O18" s="9">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>9.5000000000000001E-2</v>
       </c>
       <c r="Q18" s="1" t="s">

</xml_diff>